<commit_message>
Normalize SRS (REQ-01..18 + NFR-01..08, fix LIne2); align System Test Report + test_hardware to final IDs
</commit_message>
<xml_diff>
--- a/B-WholeSystem/docs/System_Test_Report.xlsx
+++ b/B-WholeSystem/docs/System_Test_Report.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="0" yWindow="0" windowWidth="28800" windowHeight="12300" tabRatio="600" firstSheet="0" activeTab="1" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Overall Test Report" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Test Cases &amp; Results" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Enums" sheetId="3" state="hidden" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Overall Test Report" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Cases &amp; Results" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Enums" sheetId="3" state="hidden" r:id="rId3"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="162913" fullCalcOnLoad="1"/>
@@ -248,14 +248,14 @@
 </file>
 
 <file path=xl/charts/chart1.xml><?xml version="1.0" encoding="utf-8"?>
-<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+<chartSpace xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
   <chart>
     <title>
       <tx>
         <rich>
-          <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
-          <a:lstStyle/>
-          <a:p>
+          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
             <a:pPr>
               <a:defRPr sz="1400" b="1" i="0" strike="noStrike" kern="1200" spc="0" baseline="0">
                 <a:solidFill>
@@ -279,16 +279,16 @@
       <layout/>
       <overlay val="0"/>
       <spPr>
-        <a:noFill/>
-        <a:ln>
+        <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:noFill/>
           <a:prstDash val="solid"/>
         </a:ln>
       </spPr>
       <txPr>
-        <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
-        <a:lstStyle/>
-        <a:p>
+        <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+        <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+        <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:pPr>
             <a:defRPr sz="1400" b="1" i="0" strike="noStrike" kern="1200" spc="0" baseline="0">
               <a:solidFill>
@@ -303,7 +303,7 @@
             </a:defRPr>
           </a:pPr>
           <a:r>
-            <a:t/>
+            <a:t>None</a:t>
           </a:r>
           <a:endParaRPr lang="en-US"/>
         </a:p>
@@ -317,7 +317,7 @@
           <idx val="0"/>
           <order val="0"/>
           <spPr>
-            <a:ln>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
               <a:prstDash val="solid"/>
             </a:ln>
           </spPr>
@@ -325,16 +325,16 @@
             <idx val="0"/>
             <bubble3D val="0"/>
             <spPr>
-              <a:solidFill>
+              <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:schemeClr val="accent1"/>
               </a:solidFill>
-              <a:ln w="25400">
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="25400">
                 <a:solidFill>
                   <a:schemeClr val="lt1"/>
                 </a:solidFill>
                 <a:prstDash val="solid"/>
               </a:ln>
-              <a:sp3d contourW="25400">
+              <a:sp3d xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" contourW="25400">
                 <contourClr rgb="00000000"/>
               </a:sp3d>
             </spPr>
@@ -343,16 +343,16 @@
             <idx val="1"/>
             <bubble3D val="0"/>
             <spPr>
-              <a:solidFill>
+              <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:schemeClr val="accent2"/>
               </a:solidFill>
-              <a:ln w="25400">
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="25400">
                 <a:solidFill>
                   <a:schemeClr val="lt1"/>
                 </a:solidFill>
                 <a:prstDash val="solid"/>
               </a:ln>
-              <a:sp3d contourW="25400">
+              <a:sp3d xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" contourW="25400">
                 <contourClr rgb="00000000"/>
               </a:sp3d>
             </spPr>
@@ -361,16 +361,16 @@
             <idx val="2"/>
             <bubble3D val="0"/>
             <spPr>
-              <a:solidFill>
+              <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:schemeClr val="accent3"/>
               </a:solidFill>
-              <a:ln w="25400">
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="25400">
                 <a:solidFill>
                   <a:schemeClr val="lt1"/>
                 </a:solidFill>
                 <a:prstDash val="solid"/>
               </a:ln>
-              <a:sp3d contourW="25400">
+              <a:sp3d xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" contourW="25400">
                 <contourClr rgb="00000000"/>
               </a:sp3d>
             </spPr>
@@ -438,16 +438,16 @@
       </layout>
       <overlay val="0"/>
       <spPr>
-        <a:noFill/>
-        <a:ln>
+        <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:noFill/>
           <a:prstDash val="solid"/>
         </a:ln>
       </spPr>
       <txPr>
-        <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
-        <a:lstStyle/>
-        <a:p>
+        <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+        <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+        <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:pPr rtl="0">
             <a:defRPr sz="1100" b="1" i="0" strike="noStrike" kern="1200" baseline="0">
               <a:solidFill>
@@ -462,7 +462,7 @@
             </a:defRPr>
           </a:pPr>
           <a:r>
-            <a:t/>
+            <a:t>None</a:t>
           </a:r>
           <a:endParaRPr lang="en-US"/>
         </a:p>
@@ -472,10 +472,10 @@
     <dispBlanksAs val="gap"/>
   </chart>
   <spPr>
-    <a:solidFill>
+    <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
       <a:schemeClr val="bg1"/>
     </a:solidFill>
-    <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+    <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="9525" cap="flat" cmpd="sng" algn="ctr">
       <a:solidFill>
         <a:schemeClr val="tx1">
           <a:lumMod val="15000"/>
@@ -490,7 +490,7 @@
 </file>
 
 <file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
-<wsDr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+<wsDr xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
   <twoCellAnchor>
     <from>
       <col>0</col>
@@ -510,9 +510,9 @@
         <cNvGraphicFramePr/>
       </nvGraphicFramePr>
       <xfrm/>
-      <a:graphic>
+      <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart r:id="rId1"/>
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
         </a:graphicData>
       </a:graphic>
     </graphicFrame>
@@ -1259,7 +1259,7 @@
       </c>
       <c r="D10" s="14" t="inlineStr">
         <is>
-          <t>REQ-0?</t>
+          <t>REQ-08</t>
         </is>
       </c>
       <c r="E10" s="14" t="inlineStr">
@@ -1303,7 +1303,7 @@
       </c>
       <c r="D11" s="14" t="inlineStr">
         <is>
-          <t>REQ-0?</t>
+          <t>REQ-09</t>
         </is>
       </c>
       <c r="E11" s="14" t="inlineStr">
@@ -1347,7 +1347,7 @@
       </c>
       <c r="D12" s="14" t="inlineStr">
         <is>
-          <t>REQ-0?</t>
+          <t>REQ-10</t>
         </is>
       </c>
       <c r="E12" s="14" t="inlineStr">
@@ -1391,7 +1391,7 @@
       </c>
       <c r="D13" s="14" t="inlineStr">
         <is>
-          <t>2.3.4</t>
+          <t>REQ-11</t>
         </is>
       </c>
       <c r="E13" s="14" t="inlineStr">
@@ -1435,7 +1435,7 @@
       </c>
       <c r="D14" s="14" t="inlineStr">
         <is>
-          <t>2.3.4</t>
+          <t>REQ-12</t>
         </is>
       </c>
       <c r="E14" s="14" t="inlineStr">
@@ -1479,7 +1479,7 @@
       </c>
       <c r="D15" s="14" t="inlineStr">
         <is>
-          <t>2.3.4</t>
+          <t>REQ-13</t>
         </is>
       </c>
       <c r="E15" s="14" t="inlineStr">
@@ -1523,7 +1523,7 @@
       </c>
       <c r="D16" s="14" t="inlineStr">
         <is>
-          <t>2.3.5</t>
+          <t>REQ-14</t>
         </is>
       </c>
       <c r="E16" s="14" t="inlineStr">
@@ -1567,7 +1567,7 @@
       </c>
       <c r="D17" s="14" t="inlineStr">
         <is>
-          <t>2.3.5</t>
+          <t>REQ-16</t>
         </is>
       </c>
       <c r="E17" s="14" t="inlineStr">
@@ -1611,7 +1611,7 @@
       </c>
       <c r="D18" s="14" t="inlineStr">
         <is>
-          <t>2.3.6</t>
+          <t>REQ-17</t>
         </is>
       </c>
       <c r="E18" s="14" t="inlineStr">
@@ -1655,7 +1655,7 @@
       </c>
       <c r="D19" s="14" t="inlineStr">
         <is>
-          <t>NFR-P1</t>
+          <t>NFR-01</t>
         </is>
       </c>
       <c r="E19" s="14" t="inlineStr">
@@ -1699,7 +1699,7 @@
       </c>
       <c r="D20" s="14" t="inlineStr">
         <is>
-          <t>NFR-P2</t>
+          <t>NFR-02</t>
         </is>
       </c>
       <c r="E20" s="14" t="inlineStr">
@@ -1743,7 +1743,7 @@
       </c>
       <c r="D21" s="14" t="inlineStr">
         <is>
-          <t>NFR-P4</t>
+          <t>NFR-05</t>
         </is>
       </c>
       <c r="E21" s="14" t="inlineStr">
@@ -1787,7 +1787,7 @@
       </c>
       <c r="D22" s="14" t="inlineStr">
         <is>
-          <t>NFR-P6</t>
+          <t>NFR-06</t>
         </is>
       </c>
       <c r="E22" s="14" t="inlineStr">
@@ -1831,7 +1831,7 @@
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>2.4.2</t>
+          <t>NFR-08</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">

</xml_diff>